<commit_message>
added the bounce email finder
</commit_message>
<xml_diff>
--- a/recipients.xlsx
+++ b/recipients.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>Mithra</t>
   </si>
@@ -48,10 +48,28 @@
     <t>amrita</t>
   </si>
   <si>
-    <t>Krishna</t>
-  </si>
-  <si>
-    <t>b_sreekrishna@av.amrita.edu</t>
+    <t>Rudra</t>
+  </si>
+  <si>
+    <t>rudrabhishekpalisetty2005@gmail.com</t>
+  </si>
+  <si>
+    <t>nikhil</t>
+  </si>
+  <si>
+    <t>gogole</t>
+  </si>
+  <si>
+    <t>nikhil@av.amrita.edu</t>
+  </si>
+  <si>
+    <t>amazon</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>test@av.amrita.edu</t>
   </si>
 </sst>
 </file>
@@ -869,7 +887,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="23.6640625" customWidth="1"/>
@@ -919,9 +937,33 @@
         <v>10</v>
       </c>
     </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1"/>
+    <hyperlink ref="C5" r:id="rId2"/>
+    <hyperlink ref="C6" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
improved bounce mails logic and added followup mail features
</commit_message>
<xml_diff>
--- a/recipients.xlsx
+++ b/recipients.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9252"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9255"/>
   </bookViews>
   <sheets>
     <sheet name="recipients" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>Mithra</t>
   </si>
@@ -70,6 +70,24 @@
   </si>
   <si>
     <t>test@av.amrita.edu</t>
+  </si>
+  <si>
+    <t>apple</t>
+  </si>
+  <si>
+    <t>hari</t>
+  </si>
+  <si>
+    <t>hari@av.amrita.edu</t>
+  </si>
+  <si>
+    <t>JPMC</t>
+  </si>
+  <si>
+    <t>Maneesh</t>
+  </si>
+  <si>
+    <t>maneesh@av.amrita.edu</t>
   </si>
 </sst>
 </file>
@@ -887,13 +905,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="23.6640625" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -904,7 +922,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -915,7 +933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -926,7 +944,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -937,7 +955,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -948,7 +966,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -957,6 +975,28 @@
       </c>
       <c r="C6" s="1" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -964,6 +1004,8 @@
     <hyperlink ref="C4" r:id="rId1"/>
     <hyperlink ref="C5" r:id="rId2"/>
     <hyperlink ref="C6" r:id="rId3"/>
+    <hyperlink ref="C7" r:id="rId4"/>
+    <hyperlink ref="C8" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>